<commit_message>
Coleta automática em 18-12-2025 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-12-2025 20:14
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-12-2025 20:14
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-12-2025 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-12-2025 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-12-2025 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>